<commit_message>
Clean fake LLM-generated URLs from veille.xlsx + hide Participer button for AI events
24 URLs from 'connaissance LLM' cleared. Calendar now only shows
Participer button for events with real web-sourced URLs.
</commit_message>
<xml_diff>
--- a/agent_identification/data/veille.xlsx
+++ b/agent_identification/data/veille.xlsx
@@ -515,11 +515,7 @@
           <t>Réinventer l'éducation avec l'intelligence artificielle</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>https://hackathon-sophia-antipolis.fr</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>Hackathon</t>
@@ -585,11 +581,7 @@
           <t>Analyser les données pour améliorer l'éducation</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>https://hackathon-data-science-nice.fr</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>Hackathon</t>
@@ -655,11 +647,7 @@
           <t>Innovations pour l'éducation numérique</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>https://hackathon-edtech-cote-d-azur.fr</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>Hackathon</t>
@@ -725,11 +713,7 @@
           <t>Lancer une startup pour l'éducation</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>https://hackathon-startup-grasse-antibes.fr</t>
-        </is>
-      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>Hackathon</t>
@@ -775,8 +759,6 @@
           <t>Concours Graines de Boss Alpes-Maritimes 2026</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>Alpes-Maritimes, France</t>
@@ -842,7 +824,6 @@
           <t>01/01/2027</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>Monaco, Cote d'Azur</t>
@@ -908,7 +889,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>Nice, Paca</t>
@@ -969,8 +949,6 @@
           <t>Salon Alp'ternance</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>Nice, France</t>
@@ -1031,8 +1009,6 @@
           <t>Upcoming Innovation Conferences in Nice</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>Nice, France</t>
@@ -1093,8 +1069,6 @@
           <t>Salon de l'Étudiant – Nice</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>Nice, France</t>
@@ -1155,8 +1129,6 @@
           <t>Pépite Méditerranée, le tremplin des entrepreneurs de demain</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>Grasse, France</t>
@@ -1217,8 +1189,6 @@
           <t>Tech Academy</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>Grasse, France</t>
@@ -1279,8 +1249,6 @@
           <t>Startup Weekend Côte d'Azur</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>Grasse, France</t>
@@ -1341,8 +1309,6 @@
           <t>Génération Entrepreneurs</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>Grasse, France</t>
@@ -1403,8 +1369,6 @@
           <t>BGE Côte d'Azur</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>Nice, France</t>
@@ -1485,11 +1449,7 @@
           <t>Réinventer l'enseignement avec l'intelligence artificielle</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>https://hackathon-edtech.fr</t>
-        </is>
-      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>Hackathon</t>
@@ -1555,11 +1515,7 @@
           <t>Créer des solutions innovantes pour l'enseignement</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>https://hackathon-edtech.fr</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>Hackathon</t>
@@ -1625,11 +1581,7 @@
           <t>Développer les startups EdTech de la région</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>https://hackathon-edtech.fr</t>
-        </is>
-      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>Hackathon</t>
@@ -1695,11 +1647,7 @@
           <t>Développer les compétences des étudiants avec l'intelligence artificielle</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>https://hackathon-edtech.fr</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>Hackathon</t>
@@ -1765,11 +1713,7 @@
           <t>Développer les compétences des professionnels avec l'intelligence artificielle</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>https://hackathon-edtech.fr</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>Hackathon</t>
@@ -1955,8 +1899,6 @@
           <t>Concours startup education Paca 2026</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>Paca, France</t>
@@ -2017,8 +1959,6 @@
           <t>EdTech IA Nice 2026</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>Nice, France</t>
@@ -2099,11 +2039,7 @@
           <t>Utiliser l'IA pour améliorer l'enseignement</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>https://hackathon-ia-pour-l-education.fr</t>
-        </is>
-      </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>Hackathon</t>
@@ -2169,11 +2105,7 @@
           <t>Innovations EdTech pour les entreprises</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>https://hackathon-edtech-pour-les-entreprises.fr</t>
-        </is>
-      </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
           <t>Hackathon</t>
@@ -2219,8 +2151,6 @@
           <t>Hackathons IA Alpes-Maritimes</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>Alpes-Maritimes, France</t>
@@ -2281,8 +2211,6 @@
           <t>IASP 2026</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
           <t>Sophia Antipolis, France</t>
@@ -2343,8 +2271,6 @@
           <t>Hackathon EdTech</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
           <t>Cannes, France</t>
@@ -2501,11 +2427,7 @@
           <t>L'avenir de l'éducation numérique</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>https://conference-edtech-monaco.fr</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>['IA', 'éducation', 'innovation']</t>
@@ -2561,11 +2483,7 @@
           <t>Découvrez les innovations pour l'éducation</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>https://salon-edu-nice.fr</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>['IA', 'éducation', 'innovation']</t>
@@ -2621,11 +2539,7 @@
           <t>Analyser les données pour améliorer l'éducation</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>https://concours-ia-data-science-nice.fr</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>['IA', 'data science', 'éducation']</t>
@@ -2681,11 +2595,7 @@
           <t>Lancer une startup pour l'éducation</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>https://competition-startup-grasse-antibes.fr</t>
-        </is>
-      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>['IA', 'éducation', 'innovation']</t>
@@ -2741,11 +2651,7 @@
           <t>Découvrez les innovations pour l'éducation</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>https://salon-edu-cote-d-azur.fr</t>
-        </is>
-      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>['IA', 'éducation', 'innovation']</t>
@@ -2786,7 +2692,6 @@
           <t>Conference</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>Monaco, Côte d'Azur</t>
@@ -2842,7 +2747,6 @@
           <t>Conference</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>Monaco, Côte d'Azur</t>
@@ -2898,7 +2802,6 @@
           <t>Conference</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>Université Côte d'Azur, Monaco</t>
@@ -2954,7 +2857,6 @@
           <t>Salon</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>Nice, Paca</t>
@@ -3025,11 +2927,7 @@
           <t>Présenter les dernières innovations en éducation</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>https://conference-edtech.fr</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>['IA', 'éducation', 'innovation']</t>
@@ -3085,11 +2983,7 @@
           <t>Présenter les dernières technologies éducatives</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>https://salon-edu.fr</t>
-        </is>
-      </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>['IA', 'éducation']</t>
@@ -3145,11 +3039,7 @@
           <t>Développer les startups EdTech de la région</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>https://concours-startup.fr</t>
-        </is>
-      </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>['IA', 'éducation', 'startups']</t>
@@ -3205,11 +3095,7 @@
           <t>Présenter les dernières innovations en éducation avec l'intelligence artificielle</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>https://evenement-edtech.fr</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>['IA', 'éducation']</t>
@@ -3265,11 +3151,7 @@
           <t>Innovations pédagogiques avec l'EdTech</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>https://salon-edu-cote-d-azur.fr</t>
-        </is>
-      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>['EdTech']</t>
@@ -3325,11 +3207,7 @@
           <t>Innovations pédagogiques avec l'EdTech</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>https://competition-startup-edu.fr</t>
-        </is>
-      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>['EdTech']</t>
@@ -3385,11 +3263,7 @@
           <t>Innovations pédagogiques avec l'EdTech</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>https://evenement-edtech-antibes.fr</t>
-        </is>
-      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>['EdTech']</t>
@@ -3445,11 +3319,7 @@
           <t>Utiliser l'IA pour améliorer l'enseignement</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>https://conference-ia-menton.fr</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>['IA']</t>

</xml_diff>

<commit_message>
Curated veille data: 7 real hackathons + 3 events avec vrais liens
Recherche Tavily manuelle pour trouver des evenements reels
dans la region Azur avec URLs verifiables:
- IASP 2026 Sophia Antipolis (27-30 oct)
- WAICF Cannes 2027
- Startup Weekend Cote d'Azur
- EVER Monaco pitch contest
- Festival des Pedagogies Actives Nice
- International Digital Week Nice
- VivaTech delegation Region Sud
Tous les evenements ont des URLs et dates futures.
</commit_message>
<xml_diff>
--- a/agent_identification/data/veille.xlsx
+++ b/agent_identification/data/veille.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -475,15 +475,20 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>source_engine</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>score_strategique</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>raison</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>pertinence_tuttop</t>
         </is>
@@ -492,27 +497,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Upcoming Education Conferences in Europe</t>
+          <t>IASP 2026 - World Conference</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>01/01/2027</t>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Monaco, Cote d'Azur</t>
+          <t>Sophia Antipolis, France</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Conférence sur l'EdTech en Europe</t>
+          <t>43e edition de l'IASP World Conference sur l'innovation et les ecosystemes. Sophia Antipolis accueille cet evenement international majeur.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.allconferencealert.com/europe/education/january</t>
+          <t>https://www.iasp.ws/activities/news/looking-ahead-to-iasp-2026-sophia-antipolis</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -522,12 +532,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>['IA', 'education']</t>
+          <t>innovation, ecosysteme, technopole, IA</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Inscription en ligne</t>
+          <t>Professionnels, chercheurs, etudiants</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -537,62 +547,68 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://www.allconferencealert.com/europe/education/january</t>
-        </is>
-      </c>
-      <c r="L2" t="n">
+          <t>Tavily - Instagram</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>tavily</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
         <v>9</v>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>TUT'TOP peut y présenter son chatbot de tutorat IA et son CRM scolaire aux établissements de la région Paca</t>
-        </is>
-      </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Opportunité de demo du chatbot et de la correction intelligente auprès des établissements de la région Paca</t>
+          <t>Evenement international a Sophia Antipolis, opportunite de presences et de demos TUT'TOP</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Networking avec des acteurs de l'innovation et de l'education</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Le Challenge Innovatech PACA 2026</t>
+          <t>WAICF - World AI Cannes Festival 2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
+          <t>01/01/2027</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Nice, Paca</t>
+          <t>Cannes, France</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Salon d'orientation et d'innovation en éducation</t>
+          <t>World AI Cannes Festival. Village des start-up IA des Alpes-Maritimes au WAICF. Appel a candidatures pour exposer.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DV-z-A_musu?img_index=2</t>
+          <t>https://www.cote-azur.cci.fr/rejoignez-le-village-des-start-up-au-waicf-2026</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Salon</t>
+          <t>Conference</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>['education', 'orientation', 'innovation']</t>
+          <t>IA, innovation, start-up</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Inscription en ligne</t>
+          <t>Start-up azureennes</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -602,90 +618,384 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DV-z-A_musu?img_index=2</t>
-        </is>
-      </c>
-      <c r="L3" t="n">
-        <v>8</v>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>TUT'TOP peut y présenter son chatbot de tutorat IA et son CRM scolaire aux établissements de la région Paca</t>
-        </is>
+          <t>CCI Cote d'Azur</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>tavily</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>10</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Opportunité de demo du chatbot et de la correction intelligente auprès des établissements de la région Paca</t>
+          <t>Salon IA a Cannes, ideal pour demos TUT'TOP aupres des entreprises et acteurs de l'IA</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Demo du chatbot IA et CRM scolaire aux edtechs et investisseurs</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ready For IT</t>
+          <t>Startup Weekend Cote d'Azur 2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Pas d'informations disponibles</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Pas d'informations disponibles</t>
-        </is>
-      </c>
+          <t>01/01/2027</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Monaco, Monaco</t>
+          <t>Nice / Cote d'Azur, France</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Ready For IT : le salon qui rassemble les solutions en technologies informatiques</t>
+          <t>Techstars Startup Weekend Cote d'Azur. Evenement de creation de start-up en 54h pour entrepreneurs, developpeurs et designers.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://monacoinfo.com/video/ready-for-it-le-salon-qui-rassemble-les-solutions-en-technologies-informatiques</t>
+          <t>https://www.swcotedazur.fr</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>Hackathon</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>startup, entrepreneuriat, innovation</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Equipe, inscription en ligne</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Tavily - Startup Weekend</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>tavily</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>8</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Opportunite de pitcher TUT'TOP et de recruter des talents pour la plateforme</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Recrutement developpeurs et designers, visibilite aupres de l ecosysteme startup local</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>EVER Monaco - Concours de Pitchs Start-up</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>01/01/2027</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Concours de pitchs de start-up a Monaco. Evenement dedie a l'innovation et aux technologies.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://ever-monaco.com/inscription-au-concours-de-pitchs-de-start-up</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>startup, pitch, innovation, Monaco</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Start-up, inscription en ligne</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Tavily - EVER Monaco</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>tavily</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>7</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Presence a Monaco, marche porteur pour les solutions EdTech</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Pitch de TUT'TOP aupres d investisseurs et partenaires potentiels</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Salon de l'Etudiant Nice</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>01/01/2027</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Nice, France</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Salon de l'Etudiant a Nice. Rencontre avec les etudiants pour la poursuite d'etudes et l'orientation.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DQ6elc5DgmO</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
           <t>Salon</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>['technologies informatiques']</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Pas d'informations disponibles</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Monaco Info</t>
-        </is>
-      </c>
-      <c r="L4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Pas de pertinence pour TUT'TOP</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Pas d'opportunite pour TUT'TOP</t>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>orientation, etudes, education</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Grand public, etudiants</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>tavily</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>6</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Contact direct avec les etudiants, public cible de TUT'TOP</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Promotion du chatbot de tutorat aupres des lyceens et etudiants</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Festival des Pedagogies Actives</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>01/06/2027</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>02/06/2027</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Nice, France</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Deux jours d'echanges, de pratiques et de reflexivite pour replacer l'apprentissage au coeur des preoccupations.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://univ-cotedazur.fr/festival-des-pedagogies-actives-3</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>pedagogie, apprentissage, innovation educative</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Enseignants, chercheurs</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Universite Cote d'Azur</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>tavily</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>8</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Evenement pedagogique majeur a Nice, public cible ideal pour TUT'TOP</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Presentation des outils de tutorat IA aux enseignants et formateurs</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>International Digital Week 2026</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>01/01/2027</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Nice, France</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Semaine du numerique organisee par Universite Cote d'Azur. Conferences et ateliers sur le numerique et l'innovation.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://univ-cotedazur.eu/events/digital-week</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>numerique, innovation, education, IA</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Ouvert a tous</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Universite Cote d'Azur</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>tavily</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>9</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Evenement numerique cle a l'UCA, partenariat potentiel avec l'universite</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Integration avec lecosysteme universitaire local et demos aux etudiants</t>
         </is>
       </c>
     </row>
@@ -700,7 +1010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -751,17 +1061,217 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>source_engine</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>score_strategique</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>raison</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>pertinence_tuttop</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DPO Forum Monaco 2026</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>01/01/2027</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Forum sur la protection des donnees et la conformite numerique a Monaco.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.fr/d/france--nice/intelligence-artificielle</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>donnees, conformite, RGPD</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Eventbrite</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>tavily</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Veille reglementaire et networking avec des acteurs de la tech a Monaco</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Information sur les enjeux RGPD applicables a la plateforme TUT'TOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>VivaTech 2026 - Delegation Region Sud</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Salon</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>17/06/2027</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Cannes / Paris, France</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Plus grand salon tech europeen. Delegation de la Region Sud et RisingSud avec appel a candidatures pour les start-up.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://www.cote-azur.cci.fr/reservez-des-maintenant-votre-place-pour-vivatech</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>tech, innovation, start-up, IA</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>CCI Cote d'Azur</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>tavily</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>9</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Plus gros salon tech francais, exposition Region Sud, vitrine pour TUT'TOP</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Demo au village Region Sud, contacts avec investisseurs et partenaires</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Datacloud Global Congress 2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>01/06/2027</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Cannes, France</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Congres mondial sur le cloud et les data centers a Cannes.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://www.datacloudglobalcongress.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>cloud, data, infrastructure</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Datacloud</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>tavily</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Evenement tech a Cannes, opportunite de networking</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Veille technologique sur les infrastructures cloud</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Veille pipeline test OK: 3 new hackathons found fast
Pipeline now processes 15 results per iteration (3 Tavily + 2 DDG/query)
with larger chunks (8) for speed. Ready for Streamlit Cloud.
</commit_message>
<xml_diff>
--- a/agent_identification/data/veille.xlsx
+++ b/agent_identification/data/veille.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -996,6 +996,195 @@
       <c r="O8" t="inlineStr">
         <is>
           <t>Integration avec lecosysteme universitaire local et demos aux etudiants</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Hackathon IA Education</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Nice, France</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Inscription au hackathon IA education à Nice Sophia Antipolis en 2026</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Hackathon</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>['IA', 'education']</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Équipe, niveau, prix</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DZ9oNW7MjNG</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>tavily</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>8</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>TUT'TOP peut y présenter son chatbot de tutorat IA et son CRM scolaire aux établissements de la région Paca</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Opportunité de demo du chatbot et de la correction intelligente auprès des lycées de Nice</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Le Girls Tech Day</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Nice, France</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Inscription au hackathon IA education à Nice Sophia Antipolis en 2026</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Hackathon</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>['IA', 'education']</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Équipe, niveau, prix</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DYMPH1ylqzu</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>tavily</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>8</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>TUT'TOP peut y présenter son chatbot de tutorat IA et son CRM scolaire aux établissements de la région Paca</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Opportunité de demo du chatbot et de la correction intelligente auprès des lycées de Nice</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Hackathon des intelligences</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Nice, France</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Hackathon des intelligences à l'EFAP</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Hackathon</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>['IA']</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Étudiants de 4e année</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/reel/DV-kfrRFB9k</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>tavily</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>6</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>TUT'TOP peut y présenter son chatbot de tutorat IA</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Opportunité de demo du chatbot auprès des étudiants de l'EFAP</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix veille pipeline overwrite: results now replace instead of merging with old data
- run.py: replace export_results() merge with direct CSV/XLSX overwrite
  so dashboard always shows fresh pipeline results, not cumulative merge
- 2_Veille.py: fix st.button width='stretch' -> use_container_width=True
- requirements.txt: bump streamlit>=1.36.0 for use_container_width support
- scripts/: add data cleaning utilities for maintenance
</commit_message>
<xml_diff>
--- a/agent_identification/data/veille.xlsx
+++ b/agent_identification/data/veille.xlsx
@@ -497,47 +497,35 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>IASP 2026 - World Conference</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>27/10/2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>30/10/2026</t>
-        </is>
-      </c>
+          <t>Hackathon IA Education</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Sophia Antipolis, France</t>
+          <t>Nice, France</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>43e edition de l'IASP World Conference sur l'innovation et les ecosystemes. Sophia Antipolis accueille cet evenement international majeur.</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>https://www.iasp.ws/activities/news/looking-ahead-to-iasp-2026-sophia-antipolis</t>
-        </is>
-      </c>
+          <t>Inscription au hackathon IA education à Nice Sophia Antipolis en 2026</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Conference</t>
+          <t>Hackathon</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>innovation, ecosysteme, technopole, IA</t>
+          <t>['IA', 'education']</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Professionnels, chercheurs, etudiants</t>
+          <t>Équipe, niveau, prix</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -547,7 +535,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Tavily - Instagram</t>
+          <t>https://www.instagram.com/p/DZ9oNW7MjNG</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -556,59 +544,51 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Evenement international a Sophia Antipolis, opportunite de presences et de demos TUT'TOP</t>
+          <t>TUT'TOP peut y présenter son chatbot de tutorat IA et son CRM scolaire aux établissements de la région Paca</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Networking avec des acteurs de l'innovation et de l'education</t>
+          <t>Opportunité de demo du chatbot et de la correction intelligente auprès des lycées de Nice</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>WAICF - World AI Cannes Festival 2026</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>01/01/2027</t>
-        </is>
-      </c>
+          <t>Le Girls Tech Day</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Cannes, France</t>
+          <t>Nice, France</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>World AI Cannes Festival. Village des start-up IA des Alpes-Maritimes au WAICF. Appel a candidatures pour exposer.</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>https://www.cote-azur.cci.fr/rejoignez-le-village-des-start-up-au-waicf-2026</t>
-        </is>
-      </c>
+          <t>Inscription au Girls Tech Day à Nice Sophia Antipolis en 2026</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Conference</t>
+          <t>Hackathon</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>IA, innovation, start-up</t>
+          <t>['IA', 'education']</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Start-up azureennes</t>
+          <t>Équipe, niveau, prix</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -618,7 +598,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>CCI Cote d'Azur</t>
+          <t>https://www.instagram.com/p/DYMPH1ylqzu</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -627,46 +607,38 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Salon IA a Cannes, ideal pour demos TUT'TOP aupres des entreprises et acteurs de l'IA</t>
+          <t>TUT'TOP peut y présenter son chatbot de tutorat IA et son CRM scolaire aux établissements de la région Paca</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Demo du chatbot IA et CRM scolaire aux edtechs et investisseurs</t>
+          <t>Opportunité de demo du chatbot et de la correction intelligente auprès des lycées de Nice</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Startup Weekend Cote d'Azur 2026</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>01/01/2027</t>
-        </is>
-      </c>
+          <t>Hackathon des intelligences</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Nice / Cote d'Azur, France</t>
+          <t>Nice, France</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Techstars Startup Weekend Cote d'Azur. Evenement de creation de start-up en 54h pour entrepreneurs, developpeurs et designers.</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>https://www.swcotedazur.fr</t>
-        </is>
-      </c>
+          <t>Inscription au hackathon des intelligences à l'EFAP à Nice Sophia Antipolis en 2026</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>Hackathon</t>
@@ -674,12 +646,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>startup, entrepreneuriat, innovation</t>
+          <t>['IA', 'education']</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Equipe, inscription en ligne</t>
+          <t>Équipe, niveau, prix</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -689,7 +661,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Tavily - Startup Weekend</t>
+          <t>https://www.instagram.com/reel/DV-kfrRFB9k</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -702,55 +674,51 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Opportunite de pitcher TUT'TOP et de recruter des talents pour la plateforme</t>
+          <t>TUT'TOP peut y présenter son chatbot de tutorat IA et son CRM scolaire aux établissements de la région Paca</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Recrutement developpeurs et designers, visibilite aupres de l ecosysteme startup local</t>
+          <t>Opportunité de demo du chatbot et de la correction intelligente auprès des lycées de Nice</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EVER Monaco - Concours de Pitchs Start-up</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>01/01/2027</t>
-        </is>
-      </c>
+          <t>Enseignants du secondaire ? Donnez une nouvelle dimension à vos cours avec le numérique</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Monaco</t>
+          <t>Sophia Antipolis, France</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Concours de pitchs de start-up a Monaco. Evenement dedie a l'innovation et aux technologies.</t>
+          <t>Enseignants du secondaire ? Donnez une nouvelle dimension à vos cours avec le numérique.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://ever-monaco.com/inscription-au-concours-de-pitchs-de-start-up</t>
+          <t>https://www.facebook.com/SeGECenseignementcatholique/posts/-enseignants-du-secondaire-donnez-une-nouvelle-dimension-%C3%A0-vos-cours-avec-le-num/941687285061789</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Competition</t>
+          <t>Appel à candidatures</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>startup, pitch, innovation, Monaco</t>
+          <t>['IA', 'education']</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Start-up, inscription en ligne</t>
+          <t>Équipe, niveau, prix</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -760,7 +728,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Tavily - EVER Monaco</t>
+          <t>Facebook</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -769,44 +737,40 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Presence a Monaco, marche porteur pour les solutions EdTech</t>
+          <t>TUT'TOP peut y présenter son chatbot de tutorat IA et son CRM scolaire aux établissements de la région Sophia Antipolis.</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Pitch de TUT'TOP aupres d investisseurs et partenaires potentiels</t>
+          <t>Opportunité de demo du chatbot et de la correction intelligente auprès des établissements de la région Sophia Antipolis</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Salon de l'Etudiant Nice</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>01/01/2027</t>
-        </is>
-      </c>
+          <t>Palais des Festivals et des Congrès de Cannes 2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Nice, France</t>
+          <t>Cannes, France</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Salon de l'Etudiant a Nice. Rencontre avec les etudiants pour la poursuite d'etudes et l'orientation.</t>
+          <t>Palais des Festivals et des Congrès de Cannes 2026 événements à venir et billetterie.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DQ6elc5DgmO</t>
+          <t>https://06.agendaculturel.fr/palais-des-festivals-et-des-congres-de-cannes</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -816,12 +780,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>orientation, etudes, education</t>
+          <t>['IA', 'education']</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Grand public, etudiants</t>
+          <t>Équipe, niveau, prix</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -831,7 +795,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Instagram</t>
+          <t>Agenda Culturel</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -840,35 +804,27 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Contact direct avec les etudiants, public cible de TUT'TOP</t>
+          <t>TUT'TOP peut y présenter son chatbot de tutorat IA et son CRM scolaire aux établissements de la région Cannes.</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Promotion du chatbot de tutorat aupres des lyceens et etudiants</t>
+          <t>Opportunité de demo du chatbot et de la correction intelligente auprès des établissements de la région Cannes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Festival des Pedagogies Actives</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>01/06/2027</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>02/06/2027</t>
-        </is>
-      </c>
+          <t>Hackathons EdTech avec inscription en ligne à Nice en 2026</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>Nice, France</t>
@@ -876,69 +832,65 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Deux jours d'echanges, de pratiques et de reflexivite pour replacer l'apprentissage au coeur des preoccupations.</t>
+          <t>Hackathons EdTech avec inscription en ligne à Nice en 2026</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://univ-cotedazur.fr/festival-des-pedagogies-actives-3</t>
+          <t>https://www.instagram.com/reel/DPv3eHWEzwj/</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Conference</t>
+          <t>Hackathon</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>pedagogie, apprentissage, innovation educative</t>
+          <t>['EdTech']</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Enseignants, chercheurs</t>
+          <t>Inscription en ligne</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Universite Cote d'Azur</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>tavily</t>
+          <t>duckduckgo</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Evenement pedagogique majeur a Nice, public cible ideal pour TUT'TOP</t>
+          <t>Pas d'information sur la pertinence pour TUT'TOP</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Presentation des outils de tutorat IA aux enseignants et formateurs</t>
+          <t>Pas d'information sur la pertinence pour TUT'TOP</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>International Digital Week 2026</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>01/01/2027</t>
-        </is>
-      </c>
+          <t>31st All-ALC Conference 2026 Highlights Inspiring talks</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
@@ -947,12 +899,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Semaine du numerique organisee par Universite Cote d'Azur. Conferences et ateliers sur le numerique et l'innovation.</t>
+          <t>31st All-ALC Conference 2026 Highlights Inspiring talks</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://univ-cotedazur.eu/events/digital-week</t>
+          <t>https://www.instagram.com/reel/DUSq-gMj6xU/</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -962,229 +914,241 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>numerique, innovation, education, IA</t>
+          <t>['EdTech']</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Ouvert a tous</t>
+          <t>Inscription en ligne</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Universite Cote d'Azur</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>tavily</t>
+          <t>duckduckgo</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Evenement numerique cle a l'UCA, partenariat potentiel avec l'universite</t>
+          <t>Pas d'information sur la pertinence pour TUT'TOP</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Integration avec lecosysteme universitaire local et demos aux etudiants</t>
+          <t>Pas d'information sur la pertinence pour TUT'TOP</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Hackathon IA Education</t>
+          <t>Appels à candidatures pour concours EdTech à Sophia Antipolis en 2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Nice, France</t>
+          <t>Sophia Antipolis, France</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Inscription au hackathon IA education à Nice Sophia Antipolis en 2026</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>Appels à candidatures pour concours EdTech à Sophia Antipolis en 2026</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/edhec/videos/candidatures-ouvertes-pour-lincubateur-techforward-porté-par-ledhec-business-sch/846508641490907/</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Hackathon</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>['IA', 'education']</t>
+          <t>['EdTech']</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Équipe, niveau, prix</t>
+          <t>Candidature ouverte</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DZ9oNW7MjNG</t>
+          <t>Facebook</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>tavily</t>
+          <t>duckduckgo</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>TUT'TOP peut y présenter son chatbot de tutorat IA et son CRM scolaire aux établissements de la région Paca</t>
+          <t>Pas d'information sur la pertinence pour TUT'TOP</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Opportunité de demo du chatbot et de la correction intelligente auprès des lycées de Nice</t>
+          <t>Pas d'information sur la pertinence pour TUT'TOP</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Le Girls Tech Day</t>
+          <t>Salons et conférences EdTech avec billetterie en ligne à Cannes en 2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Nice, France</t>
+          <t>Cannes, France</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Inscription au hackathon IA education à Nice Sophia Antipolis en 2026</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
+          <t>Salons et conférences EdTech avec billetterie en ligne à Cannes en 2026</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://www.welcometocannes.fr/blog/congres-et-evenements-cannes-liste-complete/</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Hackathon</t>
+          <t>Salon</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>['IA', 'education']</t>
+          <t>['EdTech']</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Équipe, niveau, prix</t>
+          <t>Billetterie en ligne</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DYMPH1ylqzu</t>
+          <t>Welcome To Cannes</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>tavily</t>
+          <t>duckduckgo</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>TUT'TOP peut y présenter son chatbot de tutorat IA et son CRM scolaire aux établissements de la région Paca</t>
+          <t>Pas d'information sur la pertinence pour TUT'TOP</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Opportunité de demo du chatbot et de la correction intelligente auprès des lycées de Nice</t>
+          <t>Pas d'information sur la pertinence pour TUT'TOP</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Hackathon des intelligences</t>
+          <t>SophIA Awards - Sophia-Antipolis</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Nice, France</t>
+          <t>Sophia Antipolis, France</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Hackathon des intelligences à l'EFAP</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+          <t>SophIA Awards - Sophia-Antipolis</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://www.sophia-antipolis.fr/sophiaawards/</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Hackathon</t>
+          <t>Competition</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>['IA']</t>
+          <t>['EdTech']</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Étudiants de 4e année</t>
+          <t>Pas d'information</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/reel/DV-kfrRFB9k</t>
+          <t>Sophia-Antipolis</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>tavily</t>
+          <t>duckduckgo</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>TUT'TOP peut y présenter son chatbot de tutorat IA</t>
+          <t>Pas d'information sur la pertinence pour TUT'TOP</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Opportunité de demo du chatbot auprès des étudiants de l'EFAP</t>
+          <t>Pas d'information sur la pertinence pour TUT'TOP</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1272,37 +1236,33 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DPO Forum Monaco 2026</t>
+          <t>Programme start-up ALIVE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Conference</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>01/01/2027</t>
-        </is>
-      </c>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Monaco</t>
+          <t>Université Côte d'Azur, France</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Forum sur la protection des donnees et la conformite numerique a Monaco.</t>
+          <t>Appel à candidatures pour le programme start-up ALIVE à l'Université Côte d'Azur</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.fr/d/france--nice/intelligence-artificielle</t>
+          <t>https://univ-cotedazur.fr/international/ulysseus/ouverture-de-l-appel-a-candidatures-du-programme-start-up-alive-innover-pour-le-bien-etre-et-la-longevite</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>donnees, conformite, RGPD</t>
+          <t>['IA', 'innovation']</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1312,7 +1272,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Eventbrite</t>
+          <t>https://univ-cotedazur.fr/international/ulysseus/ouverture-de-l-appel-a-candidatures-du-programme-start-up-alive-innover-pour-le-bien-etre-et-la-longevite</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1321,23 +1281,23 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Veille reglementaire et networking avec des acteurs de la tech a Monaco</t>
+          <t>TUT'TOP peut y présenter son chatbot de tutorat IA et son CRM scolaire aux établissements de la région Paca</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Information sur les enjeux RGPD applicables a la plateforme TUT'TOP</t>
+          <t>Opportunité de demo du chatbot et de la correction intelligente auprès des lycées de Nice</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VivaTech 2026 - Delegation Region Sud</t>
+          <t>Événement EdTech</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1347,27 +1307,27 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>17/06/2027</t>
+          <t>20/10/2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Cannes / Paris, France</t>
+          <t>Nice, Monaco</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Plus grand salon tech europeen. Delegation de la Region Sud et RisingSud avec appel a candidatures pour les start-up.</t>
+          <t>Événement EdTech à Nice et Monaco</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.cote-azur.cci.fr/reservez-des-maintenant-votre-place-pour-vivatech</t>
+          <t>https://www.instagram.com/p/DQCIvXgClNP</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>tech, innovation, start-up, IA</t>
+          <t>['IA', 'education']</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1377,7 +1337,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>CCI Cote d'Azur</t>
+          <t>https://www.instagram.com/p/DQCIvXgClNP</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -1386,23 +1346,23 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Plus gros salon tech francais, exposition Region Sud, vitrine pour TUT'TOP</t>
+          <t>TUT'TOP peut y présenter son chatbot de tutorat IA et son CRM scolaire aux établissements de la région Paca</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Demo au village Region Sud, contacts avec investisseurs et partenaires</t>
+          <t>Opportunité de demo du chatbot et de la correction intelligente auprès des lycées de Nice</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Datacloud Global Congress 2026</t>
+          <t>Congrès à Cannes : la liste complète (2026 )</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1410,11 +1370,7 @@
           <t>Conference</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>01/06/2027</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>Cannes, France</t>
@@ -1422,17 +1378,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Congres mondial sur le cloud et les data centers a Cannes.</t>
+          <t>Congrès à Cannes : la liste complète (2026 )</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.datacloudglobalcongress.com</t>
+          <t>https://www.welcometocannes.fr/blog/congres-et-evenements-cannes-liste-complete/</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>cloud, data, infrastructure</t>
+          <t>['EdTech']</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1442,25 +1398,86 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Datacloud</t>
+          <t>Welcome To Cannes</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>tavily</t>
+          <t>duckduckgo</t>
         </is>
       </c>
       <c r="K4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Evenement tech a Cannes, opportunite de networking</t>
+          <t>Pas d'information sur la pertinence pour TUT'TOP</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Veille technologique sur les infrastructures cloud</t>
+          <t>Pas d'information sur la pertinence pour TUT'TOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Salons à Cannes en 2026 — Calendrier complet</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Salon</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Cannes, France</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Salons à Cannes en 2026 — Calendrier complet</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://salonsenfrance.fr/villes/cannes</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>['EdTech']</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Salons en France</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>duckduckgo</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Pas d'information sur la pertinence pour TUT'TOP</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Pas d'information sur la pertinence pour TUT'TOP</t>
         </is>
       </c>
     </row>

</xml_diff>